<commit_message>
tests new visualize saliency
</commit_message>
<xml_diff>
--- a/results/results.xlsx
+++ b/results/results.xlsx
@@ -450,10 +450,10 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>0.2381611466407776</v>
+        <v>0.3352309465408325</v>
       </c>
     </row>
     <row r="3">
@@ -461,10 +461,10 @@
         <v>0</v>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>0.1787420362234116</v>
+        <v>0.3035429418087006</v>
       </c>
     </row>
     <row r="4">
@@ -475,7 +475,7 @@
         <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>0.1670990735292435</v>
+        <v>0.294698178768158</v>
       </c>
     </row>
     <row r="5">
@@ -483,10 +483,10 @@
         <v>0</v>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C5" t="n">
-        <v>0.1998955905437469</v>
+        <v>0.3082067370414734</v>
       </c>
     </row>
     <row r="6">
@@ -494,10 +494,10 @@
         <v>0</v>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C6" t="n">
-        <v>0.1901446431875229</v>
+        <v>0.3024156391620636</v>
       </c>
     </row>
     <row r="7">
@@ -505,10 +505,10 @@
         <v>0</v>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C7" t="n">
-        <v>0.2176174372434616</v>
+        <v>0.3188870251178741</v>
       </c>
     </row>
     <row r="8">
@@ -519,7 +519,7 @@
         <v>0</v>
       </c>
       <c r="C8" t="n">
-        <v>0.1806866824626923</v>
+        <v>0.2729175388813019</v>
       </c>
     </row>
     <row r="9">
@@ -527,10 +527,10 @@
         <v>0</v>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C9" t="n">
-        <v>0.2380498945713043</v>
+        <v>0.3027096390724182</v>
       </c>
     </row>
     <row r="10">
@@ -538,10 +538,10 @@
         <v>0</v>
       </c>
       <c r="B10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C10" t="n">
-        <v>0.233338475227356</v>
+        <v>0.3008955419063568</v>
       </c>
     </row>
     <row r="11">
@@ -549,10 +549,10 @@
         <v>0</v>
       </c>
       <c r="B11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C11" t="n">
-        <v>0.2632879316806793</v>
+        <v>0.3119738101959229</v>
       </c>
     </row>
     <row r="12">
@@ -560,10 +560,10 @@
         <v>0</v>
       </c>
       <c r="B12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C12" t="n">
-        <v>0.267630010843277</v>
+        <v>0.3028473854064941</v>
       </c>
     </row>
     <row r="13">
@@ -574,7 +574,7 @@
         <v>0</v>
       </c>
       <c r="C13" t="n">
-        <v>0.2703481614589691</v>
+        <v>0.2963594794273376</v>
       </c>
     </row>
     <row r="14">
@@ -585,7 +585,7 @@
         <v>0</v>
       </c>
       <c r="C14" t="n">
-        <v>0.2591722309589386</v>
+        <v>0.2799627482891083</v>
       </c>
     </row>
     <row r="15">
@@ -593,10 +593,10 @@
         <v>0</v>
       </c>
       <c r="B15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C15" t="n">
-        <v>0.2866141200065613</v>
+        <v>0.3011156320571899</v>
       </c>
     </row>
     <row r="16">
@@ -604,10 +604,10 @@
         <v>0</v>
       </c>
       <c r="B16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C16" t="n">
-        <v>0.2840158939361572</v>
+        <v>0.3097865581512451</v>
       </c>
     </row>
     <row r="17">
@@ -618,7 +618,7 @@
         <v>1</v>
       </c>
       <c r="C17" t="n">
-        <v>0.329104870557785</v>
+        <v>0.3424755930900574</v>
       </c>
     </row>
     <row r="18">
@@ -629,7 +629,7 @@
         <v>1</v>
       </c>
       <c r="C18" t="n">
-        <v>0.3149282336235046</v>
+        <v>0.3291063606739044</v>
       </c>
     </row>
     <row r="19">
@@ -637,10 +637,10 @@
         <v>0</v>
       </c>
       <c r="B19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C19" t="n">
-        <v>0.2867178618907928</v>
+        <v>0.3277017176151276</v>
       </c>
     </row>
     <row r="20">
@@ -651,7 +651,7 @@
         <v>1</v>
       </c>
       <c r="C20" t="n">
-        <v>0.3245745003223419</v>
+        <v>0.3446286618709564</v>
       </c>
     </row>
     <row r="21">
@@ -659,10 +659,10 @@
         <v>0</v>
       </c>
       <c r="B21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C21" t="n">
-        <v>0.2630676925182343</v>
+        <v>0.3140000402927399</v>
       </c>
     </row>
     <row r="22">
@@ -670,10 +670,10 @@
         <v>0</v>
       </c>
       <c r="B22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C22" t="n">
-        <v>0.2354423701763153</v>
+        <v>0.3034732341766357</v>
       </c>
     </row>
     <row r="23">
@@ -681,10 +681,10 @@
         <v>0</v>
       </c>
       <c r="B23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C23" t="n">
-        <v>0.2352105975151062</v>
+        <v>0.3103814721107483</v>
       </c>
     </row>
     <row r="24">
@@ -692,10 +692,10 @@
         <v>0</v>
       </c>
       <c r="B24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C24" t="n">
-        <v>0.2326998710632324</v>
+        <v>0.3156424462795258</v>
       </c>
     </row>
     <row r="25">
@@ -703,10 +703,10 @@
         <v>0</v>
       </c>
       <c r="B25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C25" t="n">
-        <v>0.2328511476516724</v>
+        <v>0.3098143637180328</v>
       </c>
     </row>
     <row r="26">
@@ -714,10 +714,10 @@
         <v>0</v>
       </c>
       <c r="B26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C26" t="n">
-        <v>0.250992476940155</v>
+        <v>0.3161989748477936</v>
       </c>
     </row>
     <row r="27">
@@ -725,10 +725,10 @@
         <v>0</v>
       </c>
       <c r="B27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C27" t="n">
-        <v>0.2467264086008072</v>
+        <v>0.3218830227851868</v>
       </c>
     </row>
     <row r="28">
@@ -736,10 +736,10 @@
         <v>0</v>
       </c>
       <c r="B28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C28" t="n">
-        <v>0.2920398712158203</v>
+        <v>0.3440283238887787</v>
       </c>
     </row>
     <row r="29">
@@ -747,10 +747,10 @@
         <v>0</v>
       </c>
       <c r="B29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C29" t="n">
-        <v>0.2850879430770874</v>
+        <v>0.3393272459506989</v>
       </c>
     </row>
     <row r="30">
@@ -758,10 +758,10 @@
         <v>0</v>
       </c>
       <c r="B30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C30" t="n">
-        <v>0.2998711168766022</v>
+        <v>0.3318997919559479</v>
       </c>
     </row>
     <row r="31">
@@ -772,7 +772,7 @@
         <v>0</v>
       </c>
       <c r="C31" t="n">
-        <v>0.215909019112587</v>
+        <v>0.2955625951290131</v>
       </c>
     </row>
     <row r="32">
@@ -783,7 +783,7 @@
         <v>0</v>
       </c>
       <c r="C32" t="n">
-        <v>0.1847217679023743</v>
+        <v>0.2794621586799622</v>
       </c>
     </row>
     <row r="33">
@@ -794,7 +794,7 @@
         <v>0</v>
       </c>
       <c r="C33" t="n">
-        <v>0.2078933864831924</v>
+        <v>0.2908841073513031</v>
       </c>
     </row>
     <row r="34">
@@ -805,7 +805,7 @@
         <v>0</v>
       </c>
       <c r="C34" t="n">
-        <v>0.2065069973468781</v>
+        <v>0.2892663776874542</v>
       </c>
     </row>
     <row r="35">
@@ -816,7 +816,7 @@
         <v>0</v>
       </c>
       <c r="C35" t="n">
-        <v>0.2093569338321686</v>
+        <v>0.2934877574443817</v>
       </c>
     </row>
     <row r="36">
@@ -824,10 +824,10 @@
         <v>0</v>
       </c>
       <c r="B36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C36" t="n">
-        <v>0.2756026089191437</v>
+        <v>0.3180401623249054</v>
       </c>
     </row>
     <row r="37">
@@ -838,7 +838,7 @@
         <v>0</v>
       </c>
       <c r="C37" t="n">
-        <v>0.1479359865188599</v>
+        <v>0.2548227906227112</v>
       </c>
     </row>
     <row r="38">
@@ -849,7 +849,7 @@
         <v>0</v>
       </c>
       <c r="C38" t="n">
-        <v>0.1436859518289566</v>
+        <v>0.2496997714042664</v>
       </c>
     </row>
     <row r="39">
@@ -860,7 +860,7 @@
         <v>0</v>
       </c>
       <c r="C39" t="n">
-        <v>0.1709278374910355</v>
+        <v>0.2598388493061066</v>
       </c>
     </row>
     <row r="40">
@@ -871,7 +871,7 @@
         <v>0</v>
       </c>
       <c r="C40" t="n">
-        <v>0.1663774102926254</v>
+        <v>0.2649215757846832</v>
       </c>
     </row>
     <row r="41">
@@ -882,7 +882,7 @@
         <v>0</v>
       </c>
       <c r="C41" t="n">
-        <v>0.1600279957056046</v>
+        <v>0.2574713230133057</v>
       </c>
     </row>
     <row r="42">
@@ -893,7 +893,7 @@
         <v>0</v>
       </c>
       <c r="C42" t="n">
-        <v>0.1752427816390991</v>
+        <v>0.270641565322876</v>
       </c>
     </row>
     <row r="43">
@@ -904,7 +904,7 @@
         <v>0</v>
       </c>
       <c r="C43" t="n">
-        <v>0.2059743702411652</v>
+        <v>0.2937043011188507</v>
       </c>
     </row>
     <row r="44">
@@ -915,7 +915,7 @@
         <v>0</v>
       </c>
       <c r="C44" t="n">
-        <v>0.2060620039701462</v>
+        <v>0.2925337851047516</v>
       </c>
     </row>
     <row r="45">
@@ -926,7 +926,7 @@
         <v>0</v>
       </c>
       <c r="C45" t="n">
-        <v>0.204648345708847</v>
+        <v>0.2909919917583466</v>
       </c>
     </row>
     <row r="46">
@@ -937,7 +937,7 @@
         <v>0</v>
       </c>
       <c r="C46" t="n">
-        <v>0.2112762182950974</v>
+        <v>0.2968530058860779</v>
       </c>
     </row>
     <row r="47">
@@ -945,10 +945,10 @@
         <v>0</v>
       </c>
       <c r="B47" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C47" t="n">
-        <v>0.2347871065139771</v>
+        <v>0.3082880675792694</v>
       </c>
     </row>
     <row r="48">
@@ -956,10 +956,10 @@
         <v>0</v>
       </c>
       <c r="B48" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C48" t="n">
-        <v>0.2617416977882385</v>
+        <v>0.3252207040786743</v>
       </c>
     </row>
     <row r="49">
@@ -967,10 +967,10 @@
         <v>0</v>
       </c>
       <c r="B49" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C49" t="n">
-        <v>0.2781640589237213</v>
+        <v>0.3309074342250824</v>
       </c>
     </row>
     <row r="50">
@@ -981,7 +981,7 @@
         <v>1</v>
       </c>
       <c r="C50" t="n">
-        <v>0.3432162702083588</v>
+        <v>0.3479488790035248</v>
       </c>
     </row>
     <row r="51">
@@ -989,10 +989,10 @@
         <v>1</v>
       </c>
       <c r="B51" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C51" t="n">
-        <v>0.2900806069374084</v>
+        <v>0.3233827948570251</v>
       </c>
     </row>
     <row r="52">
@@ -1003,7 +1003,7 @@
         <v>1</v>
       </c>
       <c r="C52" t="n">
-        <v>0.3090868890285492</v>
+        <v>0.3277689218521118</v>
       </c>
     </row>
     <row r="53">
@@ -1014,7 +1014,7 @@
         <v>1</v>
       </c>
       <c r="C53" t="n">
-        <v>0.3024193048477173</v>
+        <v>0.3276373744010925</v>
       </c>
     </row>
     <row r="54">
@@ -1025,7 +1025,7 @@
         <v>1</v>
       </c>
       <c r="C54" t="n">
-        <v>0.3328604698181152</v>
+        <v>0.3342135548591614</v>
       </c>
     </row>
     <row r="55">
@@ -1033,10 +1033,10 @@
         <v>1</v>
       </c>
       <c r="B55" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C55" t="n">
-        <v>0.2865410447120667</v>
+        <v>0.3031619787216187</v>
       </c>
     </row>
     <row r="56">
@@ -1047,7 +1047,7 @@
         <v>0</v>
       </c>
       <c r="C56" t="n">
-        <v>0.2838022112846375</v>
+        <v>0.2900123298168182</v>
       </c>
     </row>
     <row r="57">
@@ -1055,10 +1055,10 @@
         <v>1</v>
       </c>
       <c r="B57" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C57" t="n">
-        <v>0.2811754941940308</v>
+        <v>0.3026149570941925</v>
       </c>
     </row>
     <row r="58">
@@ -1069,7 +1069,7 @@
         <v>1</v>
       </c>
       <c r="C58" t="n">
-        <v>0.3058517277240753</v>
+        <v>0.3129000067710876</v>
       </c>
     </row>
     <row r="59">
@@ -1080,7 +1080,7 @@
         <v>1</v>
       </c>
       <c r="C59" t="n">
-        <v>0.3377606272697449</v>
+        <v>0.3313346207141876</v>
       </c>
     </row>
     <row r="60">
@@ -1091,7 +1091,7 @@
         <v>0</v>
       </c>
       <c r="C60" t="n">
-        <v>0.2847247719764709</v>
+        <v>0.2981729209423065</v>
       </c>
     </row>
     <row r="61">
@@ -1102,7 +1102,7 @@
         <v>0</v>
       </c>
       <c r="C61" t="n">
-        <v>0.2690600156784058</v>
+        <v>0.293770968914032</v>
       </c>
     </row>
     <row r="62">
@@ -1113,7 +1113,7 @@
         <v>0</v>
       </c>
       <c r="C62" t="n">
-        <v>0.2388896495103836</v>
+        <v>0.2746015191078186</v>
       </c>
     </row>
     <row r="63">
@@ -1124,7 +1124,7 @@
         <v>0</v>
       </c>
       <c r="C63" t="n">
-        <v>0.2653325200080872</v>
+        <v>0.2845931053161621</v>
       </c>
     </row>
     <row r="64">
@@ -1135,7 +1135,7 @@
         <v>0</v>
       </c>
       <c r="C64" t="n">
-        <v>0.2902161478996277</v>
+        <v>0.2987082302570343</v>
       </c>
     </row>
     <row r="65">
@@ -1146,7 +1146,7 @@
         <v>0</v>
       </c>
       <c r="C65" t="n">
-        <v>0.2721323668956757</v>
+        <v>0.299798846244812</v>
       </c>
     </row>
     <row r="66">
@@ -1154,10 +1154,10 @@
         <v>0</v>
       </c>
       <c r="B66" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C66" t="n">
-        <v>0.2728770077228546</v>
+        <v>0.3095797300338745</v>
       </c>
     </row>
     <row r="67">
@@ -1165,10 +1165,10 @@
         <v>0</v>
       </c>
       <c r="B67" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C67" t="n">
-        <v>0.2855453491210938</v>
+        <v>0.3127874135971069</v>
       </c>
     </row>
     <row r="68">
@@ -1176,10 +1176,10 @@
         <v>0</v>
       </c>
       <c r="B68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C68" t="n">
-        <v>0.2911399900913239</v>
+        <v>0.3111320436000824</v>
       </c>
     </row>
     <row r="69">
@@ -1190,7 +1190,7 @@
         <v>0</v>
       </c>
       <c r="C69" t="n">
-        <v>0.2712695002555847</v>
+        <v>0.2881104946136475</v>
       </c>
     </row>
     <row r="70">
@@ -1201,7 +1201,7 @@
         <v>0</v>
       </c>
       <c r="C70" t="n">
-        <v>0.2747787833213806</v>
+        <v>0.2853088676929474</v>
       </c>
     </row>
     <row r="71">
@@ -1212,7 +1212,7 @@
         <v>0</v>
       </c>
       <c r="C71" t="n">
-        <v>0.2665007710456848</v>
+        <v>0.2779954075813293</v>
       </c>
     </row>
     <row r="72">
@@ -1223,7 +1223,7 @@
         <v>0</v>
       </c>
       <c r="C72" t="n">
-        <v>0.1918675750494003</v>
+        <v>0.2919917106628418</v>
       </c>
     </row>
     <row r="73">
@@ -1234,7 +1234,7 @@
         <v>0</v>
       </c>
       <c r="C73" t="n">
-        <v>0.1737677901983261</v>
+        <v>0.2728104889392853</v>
       </c>
     </row>
     <row r="74">
@@ -1245,7 +1245,7 @@
         <v>0</v>
       </c>
       <c r="C74" t="n">
-        <v>0.1479853838682175</v>
+        <v>0.289881557226181</v>
       </c>
     </row>
     <row r="75">
@@ -1253,10 +1253,10 @@
         <v>0</v>
       </c>
       <c r="B75" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C75" t="n">
-        <v>0.1789795756340027</v>
+        <v>0.3000385165214539</v>
       </c>
     </row>
     <row r="76">
@@ -1267,7 +1267,7 @@
         <v>0</v>
       </c>
       <c r="C76" t="n">
-        <v>0.1836605817079544</v>
+        <v>0.2966263592243195</v>
       </c>
     </row>
     <row r="77">
@@ -1275,10 +1275,10 @@
         <v>0</v>
       </c>
       <c r="B77" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C77" t="n">
-        <v>0.1925239711999893</v>
+        <v>0.3012711703777313</v>
       </c>
     </row>
     <row r="78">
@@ -1289,7 +1289,7 @@
         <v>0</v>
       </c>
       <c r="C78" t="n">
-        <v>0.1849002838134766</v>
+        <v>0.289389580488205</v>
       </c>
     </row>
     <row r="79">
@@ -1300,7 +1300,7 @@
         <v>0</v>
       </c>
       <c r="C79" t="n">
-        <v>0.1963022649288177</v>
+        <v>0.2870491147041321</v>
       </c>
     </row>
     <row r="80">
@@ -1311,7 +1311,7 @@
         <v>0</v>
       </c>
       <c r="C80" t="n">
-        <v>0.2002702206373215</v>
+        <v>0.2825881838798523</v>
       </c>
     </row>
     <row r="81">
@@ -1322,7 +1322,7 @@
         <v>0</v>
       </c>
       <c r="C81" t="n">
-        <v>0.1829532980918884</v>
+        <v>0.2780455052852631</v>
       </c>
     </row>
     <row r="82">
@@ -1330,10 +1330,10 @@
         <v>0</v>
       </c>
       <c r="B82" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C82" t="n">
-        <v>0.2174079418182373</v>
+        <v>0.3147576153278351</v>
       </c>
     </row>
     <row r="83">
@@ -1344,7 +1344,7 @@
         <v>0</v>
       </c>
       <c r="C83" t="n">
-        <v>0.2201119661331177</v>
+        <v>0.2908229529857635</v>
       </c>
     </row>
     <row r="84">
@@ -1355,7 +1355,7 @@
         <v>0</v>
       </c>
       <c r="C84" t="n">
-        <v>0.2117030024528503</v>
+        <v>0.2988648116588593</v>
       </c>
     </row>
     <row r="85">
@@ -1366,7 +1366,7 @@
         <v>0</v>
       </c>
       <c r="C85" t="n">
-        <v>0.1800681352615356</v>
+        <v>0.2763010561466217</v>
       </c>
     </row>
     <row r="86">
@@ -1377,7 +1377,7 @@
         <v>0</v>
       </c>
       <c r="C86" t="n">
-        <v>0.1816184669733047</v>
+        <v>0.274865448474884</v>
       </c>
     </row>
     <row r="87">
@@ -1385,10 +1385,10 @@
         <v>0</v>
       </c>
       <c r="B87" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C87" t="n">
-        <v>0.2291494756937027</v>
+        <v>0.306006908416748</v>
       </c>
     </row>
     <row r="88">
@@ -1399,7 +1399,7 @@
         <v>0</v>
       </c>
       <c r="C88" t="n">
-        <v>0.2050115913152695</v>
+        <v>0.2927651703357697</v>
       </c>
     </row>
     <row r="89">
@@ -1410,7 +1410,7 @@
         <v>0</v>
       </c>
       <c r="C89" t="n">
-        <v>0.2024649381637573</v>
+        <v>0.2948606014251709</v>
       </c>
     </row>
     <row r="90">
@@ -1418,10 +1418,10 @@
         <v>0</v>
       </c>
       <c r="B90" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C90" t="n">
-        <v>0.2179196774959564</v>
+        <v>0.3077526390552521</v>
       </c>
     </row>
     <row r="91">
@@ -1429,10 +1429,10 @@
         <v>0</v>
       </c>
       <c r="B91" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C91" t="n">
-        <v>0.2412390112876892</v>
+        <v>0.3265544474124908</v>
       </c>
     </row>
     <row r="92">
@@ -1440,10 +1440,10 @@
         <v>0</v>
       </c>
       <c r="B92" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C92" t="n">
-        <v>0.2399351000785828</v>
+        <v>0.3268657326698303</v>
       </c>
     </row>
     <row r="93">
@@ -1454,7 +1454,7 @@
         <v>0</v>
       </c>
       <c r="C93" t="n">
-        <v>0.1864273548126221</v>
+        <v>0.2630378603935242</v>
       </c>
     </row>
     <row r="94">
@@ -1462,10 +1462,10 @@
         <v>0</v>
       </c>
       <c r="B94" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C94" t="n">
-        <v>0.2245163917541504</v>
+        <v>0.3075506985187531</v>
       </c>
     </row>
     <row r="95">
@@ -1473,10 +1473,10 @@
         <v>0</v>
       </c>
       <c r="B95" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C95" t="n">
-        <v>0.2291391640901566</v>
+        <v>0.3267741799354553</v>
       </c>
     </row>
     <row r="96">
@@ -1487,7 +1487,7 @@
         <v>0</v>
       </c>
       <c r="C96" t="n">
-        <v>0.1873904466629028</v>
+        <v>0.2662570178508759</v>
       </c>
     </row>
     <row r="97">
@@ -1498,7 +1498,7 @@
         <v>0</v>
       </c>
       <c r="C97" t="n">
-        <v>0.2067117542028427</v>
+        <v>0.2542386054992676</v>
       </c>
     </row>
     <row r="98">
@@ -1509,7 +1509,7 @@
         <v>1</v>
       </c>
       <c r="C98" t="n">
-        <v>0.3241853713989258</v>
+        <v>0.3390501737594604</v>
       </c>
     </row>
     <row r="99">
@@ -1520,7 +1520,7 @@
         <v>0</v>
       </c>
       <c r="C99" t="n">
-        <v>0.2102421075105667</v>
+        <v>0.2899646759033203</v>
       </c>
     </row>
     <row r="100">
@@ -1528,10 +1528,10 @@
         <v>0</v>
       </c>
       <c r="B100" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C100" t="n">
-        <v>0.2318217903375626</v>
+        <v>0.3000012636184692</v>
       </c>
     </row>
     <row r="101">
@@ -1542,7 +1542,7 @@
         <v>0</v>
       </c>
       <c r="C101" t="n">
-        <v>0.2403066158294678</v>
+        <v>0.2996857166290283</v>
       </c>
     </row>
     <row r="102">
@@ -1553,7 +1553,7 @@
         <v>0</v>
       </c>
       <c r="C102" t="n">
-        <v>0.2399089932441711</v>
+        <v>0.295087605714798</v>
       </c>
     </row>
     <row r="103">
@@ -1564,7 +1564,7 @@
         <v>0</v>
       </c>
       <c r="C103" t="n">
-        <v>0.2295450270175934</v>
+        <v>0.2896869480609894</v>
       </c>
     </row>
     <row r="104">
@@ -1575,7 +1575,7 @@
         <v>0</v>
       </c>
       <c r="C104" t="n">
-        <v>0.2405727505683899</v>
+        <v>0.2927162349224091</v>
       </c>
     </row>
     <row r="105">
@@ -1586,7 +1586,7 @@
         <v>0</v>
       </c>
       <c r="C105" t="n">
-        <v>0.24461829662323</v>
+        <v>0.2937803864479065</v>
       </c>
     </row>
     <row r="106">
@@ -1597,7 +1597,7 @@
         <v>0</v>
       </c>
       <c r="C106" t="n">
-        <v>0.2224791795015335</v>
+        <v>0.2852213978767395</v>
       </c>
     </row>
     <row r="107">
@@ -1608,7 +1608,7 @@
         <v>0</v>
       </c>
       <c r="C107" t="n">
-        <v>0.2433880269527435</v>
+        <v>0.2994324266910553</v>
       </c>
     </row>
     <row r="108">
@@ -1616,10 +1616,10 @@
         <v>0</v>
       </c>
       <c r="B108" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C108" t="n">
-        <v>0.24950310587883</v>
+        <v>0.3076993227005005</v>
       </c>
     </row>
     <row r="109">
@@ -1627,10 +1627,10 @@
         <v>0</v>
       </c>
       <c r="B109" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C109" t="n">
-        <v>0.2988097369670868</v>
+        <v>0.3363834619522095</v>
       </c>
     </row>
     <row r="110">
@@ -1641,7 +1641,7 @@
         <v>0</v>
       </c>
       <c r="C110" t="n">
-        <v>0.1433841437101364</v>
+        <v>0.2768828868865967</v>
       </c>
     </row>
     <row r="111">
@@ -1652,7 +1652,7 @@
         <v>0</v>
       </c>
       <c r="C111" t="n">
-        <v>0.1670248061418533</v>
+        <v>0.2923911511898041</v>
       </c>
     </row>
     <row r="112">
@@ -1663,7 +1663,7 @@
         <v>0</v>
       </c>
       <c r="C112" t="n">
-        <v>0.1804302483797073</v>
+        <v>0.2901846170425415</v>
       </c>
     </row>
     <row r="113">
@@ -1674,7 +1674,7 @@
         <v>0</v>
       </c>
       <c r="C113" t="n">
-        <v>0.1787750273942947</v>
+        <v>0.2920569777488708</v>
       </c>
     </row>
     <row r="114">
@@ -1685,7 +1685,7 @@
         <v>0</v>
       </c>
       <c r="C114" t="n">
-        <v>0.1716841161251068</v>
+        <v>0.2816106379032135</v>
       </c>
     </row>
     <row r="115">
@@ -1696,7 +1696,7 @@
         <v>0</v>
       </c>
       <c r="C115" t="n">
-        <v>0.1638062596321106</v>
+        <v>0.282250702381134</v>
       </c>
     </row>
     <row r="116">
@@ -1704,10 +1704,10 @@
         <v>0</v>
       </c>
       <c r="B116" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C116" t="n">
-        <v>0.1949034333229065</v>
+        <v>0.3100714981555939</v>
       </c>
     </row>
     <row r="117">
@@ -1715,10 +1715,10 @@
         <v>0</v>
       </c>
       <c r="B117" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C117" t="n">
-        <v>0.1934078484773636</v>
+        <v>0.3105649948120117</v>
       </c>
     </row>
     <row r="118">
@@ -1726,10 +1726,10 @@
         <v>0</v>
       </c>
       <c r="B118" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C118" t="n">
-        <v>0.2255610972642899</v>
+        <v>0.3286233246326447</v>
       </c>
     </row>
     <row r="119">
@@ -1737,10 +1737,10 @@
         <v>0</v>
       </c>
       <c r="B119" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C119" t="n">
-        <v>0.2226466983556747</v>
+        <v>0.3316271007061005</v>
       </c>
     </row>
     <row r="120">
@@ -1751,7 +1751,7 @@
         <v>0</v>
       </c>
       <c r="C120" t="n">
-        <v>0.2166190147399902</v>
+        <v>0.2713590860366821</v>
       </c>
     </row>
     <row r="121">
@@ -1759,10 +1759,10 @@
         <v>1</v>
       </c>
       <c r="B121" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C121" t="n">
-        <v>0.2742612957954407</v>
+        <v>0.3124756813049316</v>
       </c>
     </row>
     <row r="122">
@@ -1770,10 +1770,10 @@
         <v>1</v>
       </c>
       <c r="B122" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C122" t="n">
-        <v>0.255401223897934</v>
+        <v>0.3046939969062805</v>
       </c>
     </row>
     <row r="123">
@@ -1784,7 +1784,7 @@
         <v>0</v>
       </c>
       <c r="C123" t="n">
-        <v>0.2767384350299835</v>
+        <v>0.2959698140621185</v>
       </c>
     </row>
     <row r="124">
@@ -1795,7 +1795,7 @@
         <v>0</v>
       </c>
       <c r="C124" t="n">
-        <v>0.2475635558366776</v>
+        <v>0.2891551852226257</v>
       </c>
     </row>
     <row r="125">
@@ -1806,7 +1806,7 @@
         <v>0</v>
       </c>
       <c r="C125" t="n">
-        <v>0.250551164150238</v>
+        <v>0.297671765089035</v>
       </c>
     </row>
     <row r="126">
@@ -1817,7 +1817,7 @@
         <v>0</v>
       </c>
       <c r="C126" t="n">
-        <v>0.249022364616394</v>
+        <v>0.2902853786945343</v>
       </c>
     </row>
     <row r="127">
@@ -1828,7 +1828,7 @@
         <v>0</v>
       </c>
       <c r="C127" t="n">
-        <v>0.2319845259189606</v>
+        <v>0.2792885303497314</v>
       </c>
     </row>
     <row r="128">
@@ -1836,10 +1836,10 @@
         <v>1</v>
       </c>
       <c r="B128" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C128" t="n">
-        <v>0.263652503490448</v>
+        <v>0.3008041679859161</v>
       </c>
     </row>
     <row r="129">
@@ -1850,7 +1850,7 @@
         <v>0</v>
       </c>
       <c r="C129" t="n">
-        <v>0.2748886346817017</v>
+        <v>0.2998161315917969</v>
       </c>
     </row>
     <row r="130">
@@ -1861,7 +1861,7 @@
         <v>0</v>
       </c>
       <c r="C130" t="n">
-        <v>0.2624746263027191</v>
+        <v>0.2919549345970154</v>
       </c>
     </row>
     <row r="131">
@@ -1869,10 +1869,10 @@
         <v>1</v>
       </c>
       <c r="B131" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C131" t="n">
-        <v>0.2701574563980103</v>
+        <v>0.3018651604652405</v>
       </c>
     </row>
     <row r="132">
@@ -1880,10 +1880,10 @@
         <v>1</v>
       </c>
       <c r="B132" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C132" t="n">
-        <v>0.2955268323421478</v>
+        <v>0.3126275241374969</v>
       </c>
     </row>
     <row r="133">
@@ -1891,10 +1891,10 @@
         <v>1</v>
       </c>
       <c r="B133" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C133" t="n">
-        <v>0.2910527884960175</v>
+        <v>0.3333138227462769</v>
       </c>
     </row>
     <row r="134">
@@ -1902,10 +1902,10 @@
         <v>0</v>
       </c>
       <c r="B134" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C134" t="n">
-        <v>0.2334237694740295</v>
+        <v>0.3117635250091553</v>
       </c>
     </row>
     <row r="135">
@@ -1913,10 +1913,10 @@
         <v>0</v>
       </c>
       <c r="B135" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C135" t="n">
-        <v>0.2364491820335388</v>
+        <v>0.3096433579921722</v>
       </c>
     </row>
     <row r="136">
@@ -1924,10 +1924,10 @@
         <v>0</v>
       </c>
       <c r="B136" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C136" t="n">
-        <v>0.2861479818820953</v>
+        <v>0.3255072832107544</v>
       </c>
     </row>
     <row r="137">
@@ -1935,10 +1935,10 @@
         <v>0</v>
       </c>
       <c r="B137" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C137" t="n">
-        <v>0.2746149599552155</v>
+        <v>0.3351421356201172</v>
       </c>
     </row>
     <row r="138">
@@ -1946,10 +1946,10 @@
         <v>0</v>
       </c>
       <c r="B138" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C138" t="n">
-        <v>0.2777868509292603</v>
+        <v>0.3301644325256348</v>
       </c>
     </row>
     <row r="139">
@@ -1957,10 +1957,10 @@
         <v>0</v>
       </c>
       <c r="B139" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C139" t="n">
-        <v>0.2663631439208984</v>
+        <v>0.316480964422226</v>
       </c>
     </row>
     <row r="140">
@@ -1968,10 +1968,10 @@
         <v>0</v>
       </c>
       <c r="B140" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C140" t="n">
-        <v>0.2583484351634979</v>
+        <v>0.3150219619274139</v>
       </c>
     </row>
     <row r="141">
@@ -1982,7 +1982,7 @@
         <v>0</v>
       </c>
       <c r="C141" t="n">
-        <v>0.2406353503465652</v>
+        <v>0.298509418964386</v>
       </c>
     </row>
     <row r="142">
@@ -1990,10 +1990,10 @@
         <v>1</v>
       </c>
       <c r="B142" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C142" t="n">
-        <v>0.2551130652427673</v>
+        <v>0.3341828286647797</v>
       </c>
     </row>
     <row r="143">
@@ -2001,10 +2001,10 @@
         <v>1</v>
       </c>
       <c r="B143" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C143" t="n">
-        <v>0.2794508635997772</v>
+        <v>0.3251211047172546</v>
       </c>
     </row>
     <row r="144">
@@ -2012,10 +2012,10 @@
         <v>1</v>
       </c>
       <c r="B144" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C144" t="n">
-        <v>0.2909943163394928</v>
+        <v>0.3219552040100098</v>
       </c>
     </row>
     <row r="145">
@@ -2023,10 +2023,10 @@
         <v>1</v>
       </c>
       <c r="B145" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C145" t="n">
-        <v>0.2944423258304596</v>
+        <v>0.3099992275238037</v>
       </c>
     </row>
     <row r="146">
@@ -2034,10 +2034,10 @@
         <v>1</v>
       </c>
       <c r="B146" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C146" t="n">
-        <v>0.2853884696960449</v>
+        <v>0.3114360868930817</v>
       </c>
     </row>
     <row r="147">
@@ -2045,10 +2045,10 @@
         <v>1</v>
       </c>
       <c r="B147" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C147" t="n">
-        <v>0.2816774845123291</v>
+        <v>0.3156703114509583</v>
       </c>
     </row>
     <row r="148">
@@ -2056,10 +2056,10 @@
         <v>1</v>
       </c>
       <c r="B148" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C148" t="n">
-        <v>0.2916271984577179</v>
+        <v>0.3240561187267303</v>
       </c>
     </row>
     <row r="149">
@@ -2067,10 +2067,10 @@
         <v>1</v>
       </c>
       <c r="B149" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C149" t="n">
-        <v>0.2839883863925934</v>
+        <v>0.3199943900108337</v>
       </c>
     </row>
     <row r="150">
@@ -2078,10 +2078,10 @@
         <v>1</v>
       </c>
       <c r="B150" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C150" t="n">
-        <v>0.2834880352020264</v>
+        <v>0.3248811960220337</v>
       </c>
     </row>
     <row r="151">
@@ -2089,10 +2089,10 @@
         <v>1</v>
       </c>
       <c r="B151" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C151" t="n">
-        <v>0.2799760699272156</v>
+        <v>0.3230020105838776</v>
       </c>
     </row>
     <row r="152">
@@ -2100,10 +2100,10 @@
         <v>1</v>
       </c>
       <c r="B152" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C152" t="n">
-        <v>0.2706081569194794</v>
+        <v>0.3184911906719208</v>
       </c>
     </row>
     <row r="153">
@@ -2111,10 +2111,10 @@
         <v>1</v>
       </c>
       <c r="B153" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C153" t="n">
-        <v>0.2615512013435364</v>
+        <v>0.3173831403255463</v>
       </c>
     </row>
     <row r="154">
@@ -2122,10 +2122,10 @@
         <v>1</v>
       </c>
       <c r="B154" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C154" t="n">
-        <v>0.2731585502624512</v>
+        <v>0.33001908659935</v>
       </c>
     </row>
   </sheetData>

</xml_diff>